<commit_message>
Updated scenario links voor 2015.1 ETM engine
Updated scenario links voor 2015.1 ETM engine.
</commit_message>
<xml_diff>
--- a/hail/data/scenario_links_grdr.xlsx
+++ b/hail/data/scenario_links_grdr.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NAVE\Documents\Lopende Projecten\TIP Groningen local\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HOUJ\Downloads\Python_2\TIP\hail\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A585414-19B0-4D8D-BFF0-7FA2CE016834}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16F264A3-E027-44A7-B822-93032DF10D48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="KM 2050" sheetId="1" r:id="rId1"/>
@@ -260,86 +260,86 @@
     <t>GM0160</t>
   </si>
   <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475562</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475564</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475566</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475567</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475568</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475569</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475570</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475572</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475573</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475574</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475575</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475576</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475577</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475578</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475580</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475581</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475582</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475583</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475584</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475585</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475586</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475587</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475588</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475589</t>
-  </si>
-  <si>
-    <t>https://pro.energytransitionmodel.com/scenarios/1475591</t>
+    <t>https://pro.energytransitionmodel.com/scenarios/90442</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90461</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90460</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90459</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90458</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90457</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90456</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90455</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90454</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90453</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90452</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90451</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90450</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90449</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90448</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90447</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90446</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90445</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90444</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90443</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90435</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90437</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90438</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90439</t>
+  </si>
+  <si>
+    <t>https://pro.energytransitionmodel.com/scenarios/90440</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -692,22 +692,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="53.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="53.28515625" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -715,13 +715,16 @@
       <c r="D1" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E1">
+        <v>90461</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
         <v>51</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C2" t="s">
         <v>1</v>
@@ -729,13 +732,16 @@
       <c r="D2" s="1" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E2">
+        <v>90460</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" s="1" t="s">
         <v>52</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C3" t="s">
         <v>2</v>
@@ -743,13 +749,16 @@
       <c r="D3" s="1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E3">
+        <v>90459</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C4" t="s">
         <v>3</v>
@@ -757,13 +766,16 @@
       <c r="D4" s="1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E4">
+        <v>90458</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5" s="1" t="s">
         <v>54</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C5" t="s">
         <v>4</v>
@@ -771,13 +783,16 @@
       <c r="D5" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E5">
+        <v>90457</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6" s="1" t="s">
         <v>55</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C6" t="s">
         <v>5</v>
@@ -785,13 +800,16 @@
       <c r="D6" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E6">
+        <v>90456</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
       <c r="A7" s="1" t="s">
         <v>56</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C7" t="s">
         <v>6</v>
@@ -799,13 +817,16 @@
       <c r="D7" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E7">
+        <v>90455</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
       <c r="A8" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C8" t="s">
         <v>7</v>
@@ -813,13 +834,16 @@
       <c r="D8" s="1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E8">
+        <v>90454</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
       <c r="A9" s="1" t="s">
         <v>58</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C9" t="s">
         <v>8</v>
@@ -827,13 +851,16 @@
       <c r="D9" s="1" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E9">
+        <v>90453</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
       <c r="A10" s="1" t="s">
         <v>59</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C10" t="s">
         <v>9</v>
@@ -841,13 +868,16 @@
       <c r="D10" s="1" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E10">
+        <v>90452</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
       <c r="A11" s="1" t="s">
         <v>60</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C11" t="s">
         <v>10</v>
@@ -855,13 +885,16 @@
       <c r="D11" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E11">
+        <v>90451</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
       <c r="A12" s="1" t="s">
         <v>61</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C12" t="s">
         <v>11</v>
@@ -869,13 +902,16 @@
       <c r="D12" s="1" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E12">
+        <v>90450</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
       <c r="A13" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C13" t="s">
         <v>12</v>
@@ -883,13 +919,16 @@
       <c r="D13" s="1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E13">
+        <v>90449</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
       <c r="A14" s="1" t="s">
         <v>63</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C14" t="s">
         <v>13</v>
@@ -897,13 +936,16 @@
       <c r="D14" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E14">
+        <v>90448</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
       <c r="A15" s="1" t="s">
         <v>64</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C15" t="s">
         <v>14</v>
@@ -911,13 +953,16 @@
       <c r="D15" s="1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E15">
+        <v>90447</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
       <c r="A16" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C16" t="s">
         <v>15</v>
@@ -925,13 +970,16 @@
       <c r="D16" s="1" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E16">
+        <v>90446</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
       <c r="A17" s="1" t="s">
         <v>66</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C17" t="s">
         <v>16</v>
@@ -939,13 +987,16 @@
       <c r="D17" s="1" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E17">
+        <v>90445</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
       <c r="A18" s="1" t="s">
         <v>67</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C18" t="s">
         <v>17</v>
@@ -953,13 +1004,16 @@
       <c r="D18" s="1" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E18">
+        <v>90444</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
       <c r="A19" s="1" t="s">
         <v>68</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C19" t="s">
         <v>18</v>
@@ -967,13 +1021,16 @@
       <c r="D19" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E19">
+        <v>90443</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
       <c r="A20" s="1" t="s">
         <v>69</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C20" t="s">
         <v>19</v>
@@ -981,13 +1038,16 @@
       <c r="D20" s="1" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E20">
+        <v>90435</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
       <c r="A21" s="1" t="s">
         <v>70</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C21" t="s">
         <v>20</v>
@@ -995,13 +1055,16 @@
       <c r="D21" s="1" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E21">
+        <v>90437</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
       <c r="A22" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C22" t="s">
         <v>21</v>
@@ -1009,13 +1072,16 @@
       <c r="D22" s="1" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E22">
+        <v>90438</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
       <c r="A23" s="1" t="s">
         <v>72</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C23" t="s">
         <v>22</v>
@@ -1023,13 +1089,16 @@
       <c r="D23" s="1" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E23">
+        <v>90439</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
       <c r="A24" s="1" t="s">
         <v>73</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C24" t="s">
         <v>23</v>
@@ -1037,13 +1106,16 @@
       <c r="D24" s="1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="E24">
+        <v>90440</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
       <c r="A25" s="1" t="s">
         <v>74</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>99</v>
+        <v>75</v>
       </c>
       <c r="C25" t="s">
         <v>24</v>
@@ -1051,34 +1123,14 @@
       <c r="D25" s="1" t="s">
         <v>49</v>
       </c>
+      <c r="E25">
+        <v>90442</v>
+      </c>
+      <c r="H25" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B1" r:id="rId1" xr:uid="{3FA1073C-0AA0-4CB6-B044-A805CCE36937}"/>
-    <hyperlink ref="B2" r:id="rId2" xr:uid="{C64287AB-F510-49E4-B8B9-40C487B6FC2F}"/>
-    <hyperlink ref="B3" r:id="rId3" xr:uid="{EF27B0F8-B168-4F05-BE9A-5E81F4285309}"/>
-    <hyperlink ref="B4" r:id="rId4" xr:uid="{A0712407-F37C-41C9-AE7E-F68F2F85D968}"/>
-    <hyperlink ref="B5" r:id="rId5" xr:uid="{2BB995B7-3DAC-48D0-8679-756C17B7B44B}"/>
-    <hyperlink ref="B6" r:id="rId6" xr:uid="{830B4FD4-9988-46B5-9340-E1217DFC386A}"/>
-    <hyperlink ref="B7" r:id="rId7" xr:uid="{78D46F14-E9B2-40A3-8F37-C2062C839DDD}"/>
-    <hyperlink ref="B8" r:id="rId8" xr:uid="{3F731592-C9F1-4534-942A-A9211C0AA8BA}"/>
-    <hyperlink ref="B9" r:id="rId9" xr:uid="{5F9E7353-037A-43CE-B32C-935FB0D75BD7}"/>
-    <hyperlink ref="B10" r:id="rId10" xr:uid="{0EB1B1A4-52E2-4941-B06E-18B973A88194}"/>
-    <hyperlink ref="B11" r:id="rId11" xr:uid="{964F92F3-3274-4C83-8FDB-0D8311A9EEAF}"/>
-    <hyperlink ref="B12" r:id="rId12" xr:uid="{6DB115FF-E5CC-410A-A663-5D9266C5D334}"/>
-    <hyperlink ref="B13" r:id="rId13" xr:uid="{1A7F5769-26FA-4A84-8645-F8007AB14292}"/>
-    <hyperlink ref="B14" r:id="rId14" xr:uid="{0C4731A5-9CD2-45EC-840C-8E97F280C381}"/>
-    <hyperlink ref="B15" r:id="rId15" xr:uid="{01E1CA4B-8F56-491D-8071-1640DBCB5F2F}"/>
-    <hyperlink ref="B16" r:id="rId16" xr:uid="{F201ED59-BD18-4A43-8861-D0A6758FD2E7}"/>
-    <hyperlink ref="B17" r:id="rId17" xr:uid="{9A3F4D2B-590D-4EAD-B3EB-CED5570D9170}"/>
-    <hyperlink ref="B18" r:id="rId18" xr:uid="{2D821685-DF6A-4EEC-BFC2-B42853222BAB}"/>
-    <hyperlink ref="B19" r:id="rId19" xr:uid="{54F886AE-75EF-42EB-B502-3CFE6FCFEB5B}"/>
-    <hyperlink ref="B20" r:id="rId20" xr:uid="{901A6F05-E83A-4B4C-9570-C356F197C611}"/>
-    <hyperlink ref="B21" r:id="rId21" xr:uid="{1071A242-140A-4772-914D-6EA6EAFC4061}"/>
-    <hyperlink ref="B22" r:id="rId22" xr:uid="{9080EC19-9E59-4973-AEB3-86D88194A116}"/>
-    <hyperlink ref="B23" r:id="rId23" xr:uid="{57AF91E6-40B5-4F1A-99D9-9330B1CCBBB3}"/>
-    <hyperlink ref="B24" r:id="rId24" xr:uid="{F1D80140-E35E-48A7-8190-539BF3CCC4F3}"/>
-    <hyperlink ref="B25" r:id="rId25" xr:uid="{CA74E4FA-5E83-4CF5-AB44-51E603D067E9}"/>
+    <hyperlink ref="B17" r:id="rId1" xr:uid="{4DB52D4D-561F-4F0B-96C1-B63FE02A0B71}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>